<commit_message>
added graph, month total per category (fix pendin)
</commit_message>
<xml_diff>
--- a/Gastos.xlsx
+++ b/Gastos.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enero" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diciembre" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -58,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -355,10 +356,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="3">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -384,8 +385,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -398,10 +499,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="3">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -427,8 +528,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -441,10 +642,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -470,8 +671,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -484,10 +785,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -513,8 +814,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
     <row r="3" ht="14.25" customHeight="1" s="3"/>
     <row r="4" ht="14.25" customHeight="1" s="3"/>
   </sheetData>
@@ -529,10 +930,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -558,8 +959,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -572,10 +1073,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -601,8 +1102,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -615,10 +1216,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -644,8 +1245,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -658,10 +1359,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -687,8 +1388,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -701,10 +1502,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -730,8 +1531,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -744,7 +1645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
@@ -780,6 +1681,61 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -805,6 +1761,50 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -876,6 +1876,31 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-07-11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -893,10 +1918,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -922,8 +1947,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -936,10 +2061,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" s="3">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -965,8 +2090,108 @@
           <t>Cuotas pendientes</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1" s="3"/>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Alquiler</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Expensas</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Bolucompra</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Ahorros</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1" s="3">
+      <c r="F2">
+        <f>SUMIF(B:B,F1,C:C)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(B:B,G1,C:C)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(B:B,H1,C:C)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(B:B,I1,C:C)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(B:B,J1,C:C)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(B:B,K1,C:C)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(B:B,L1,C:C)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIF(B:B,M1,C:C)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIF(B:B,N1,C:C)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(B:B,O1,C:C)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUMIF(B:B,P1,C:C)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>